<commit_message>
chore: fresh runs of vfvv, investigating optimal dvs intervals
</commit_message>
<xml_diff>
--- a/excel/CombinedEfficiencyStats.xlsx
+++ b/excel/CombinedEfficiencyStats.xlsx
@@ -495,28 +495,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>42.6682</v>
+        <v>42.7863</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0294678</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>42.7173</v>
+        <v>42.7863</v>
       </c>
       <c r="F2" t="n">
         <v>356.67</v>
       </c>
       <c r="G2" t="n">
-        <v>357.24</v>
+        <v>359.84</v>
       </c>
       <c r="H2" t="n">
-        <v>343.359</v>
+        <v>341.116</v>
       </c>
       <c r="I2" t="n">
-        <v>343.393</v>
+        <v>341.179</v>
       </c>
       <c r="J2" t="n">
-        <v>21084100000</v>
+        <v>21102200000</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -539,28 +539,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.458</v>
+        <v>42.5422</v>
       </c>
       <c r="D3" t="n">
-        <v>0.018281</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>42.4914</v>
+        <v>42.5422</v>
       </c>
       <c r="F3" t="n">
         <v>356.66</v>
       </c>
       <c r="G3" t="n">
-        <v>357.18</v>
+        <v>359.84</v>
       </c>
       <c r="H3" t="n">
-        <v>343.181</v>
+        <v>339.448</v>
       </c>
       <c r="I3" t="n">
-        <v>343.183</v>
+        <v>339.464</v>
       </c>
       <c r="J3" t="n">
-        <v>31107500000</v>
+        <v>31125600000</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -680,16 +680,16 @@
         <v>42.6729</v>
       </c>
       <c r="F6" t="n">
-        <v>354.79</v>
+        <v>355.89</v>
       </c>
       <c r="G6" t="n">
-        <v>357.83</v>
+        <v>359.16</v>
       </c>
       <c r="H6" t="n">
-        <v>344.184</v>
+        <v>344.864</v>
       </c>
       <c r="I6" t="n">
-        <v>344.471</v>
+        <v>345.268</v>
       </c>
       <c r="J6" t="n">
         <v>11393400000</v>
@@ -759,28 +759,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>41.3974</v>
+        <v>42.0503</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>41.3974</v>
+        <v>42.0503</v>
       </c>
       <c r="F8" t="n">
-        <v>353.76</v>
+        <v>360.62</v>
       </c>
       <c r="G8" t="n">
-        <v>356.26</v>
+        <v>371.4</v>
       </c>
       <c r="H8" t="n">
-        <v>351.215</v>
+        <v>332.508</v>
       </c>
       <c r="I8" t="n">
-        <v>351.445</v>
+        <v>333.229</v>
       </c>
       <c r="J8" t="n">
-        <v>108753000</v>
+        <v>53270600000</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -803,28 +803,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>39.0663</v>
+        <v>39.7091</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0442546</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>39.2443</v>
+        <v>39.7091</v>
       </c>
       <c r="F9" t="n">
         <v>355.59</v>
       </c>
       <c r="G9" t="n">
-        <v>357.28</v>
+        <v>358.56</v>
       </c>
       <c r="H9" t="n">
         <v>345.336</v>
       </c>
       <c r="I9" t="n">
-        <v>345.295</v>
+        <v>345.32</v>
       </c>
       <c r="J9" t="n">
-        <v>7428300000</v>
+        <v>7450060000</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -856,16 +856,16 @@
         <v>41.1417</v>
       </c>
       <c r="F10" t="n">
-        <v>353.5</v>
+        <v>355.68</v>
       </c>
       <c r="G10" t="n">
-        <v>355.79</v>
+        <v>358.51</v>
       </c>
       <c r="H10" t="n">
-        <v>351.229</v>
+        <v>352.041</v>
       </c>
       <c r="I10" t="n">
-        <v>351.432</v>
+        <v>352.392</v>
       </c>
       <c r="J10" t="n">
         <v>226227000</v>
@@ -979,28 +979,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-52.4796</v>
+        <v>40.6204</v>
       </c>
       <c r="D13" t="n">
-        <v>-4.81295</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>-2.38932</v>
+        <v>40.6204</v>
       </c>
       <c r="F13" t="n">
         <v>356.3</v>
       </c>
       <c r="G13" t="n">
-        <v>357.29</v>
+        <v>362.28</v>
       </c>
       <c r="H13" t="n">
         <v>332.99</v>
       </c>
       <c r="I13" t="n">
-        <v>331.573</v>
+        <v>333.295</v>
       </c>
       <c r="J13" t="n">
-        <v>59637200000</v>
+        <v>88812600000</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1111,28 +1111,28 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>53.8296</v>
+        <v>53.9247</v>
       </c>
       <c r="D16" t="n">
-        <v>20.0354</v>
+        <v>20</v>
       </c>
       <c r="E16" t="n">
-        <v>44.643</v>
+        <v>44.7097</v>
       </c>
       <c r="F16" t="n">
         <v>357.41</v>
       </c>
       <c r="G16" t="n">
-        <v>357.24</v>
+        <v>359.84</v>
       </c>
       <c r="H16" t="n">
-        <v>344.422</v>
+        <v>342.391</v>
       </c>
       <c r="I16" t="n">
-        <v>343.393</v>
+        <v>341.179</v>
       </c>
       <c r="J16" t="n">
-        <v>21084100000</v>
+        <v>21102200000</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1155,28 +1155,28 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>53.7875</v>
+        <v>53.8552</v>
       </c>
       <c r="D17" t="n">
-        <v>20.0219</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
-        <v>44.5772</v>
+        <v>44.6262</v>
       </c>
       <c r="F17" t="n">
         <v>357.39</v>
       </c>
       <c r="G17" t="n">
-        <v>357.18</v>
+        <v>359.84</v>
       </c>
       <c r="H17" t="n">
-        <v>344.239</v>
+        <v>340.784</v>
       </c>
       <c r="I17" t="n">
-        <v>343.183</v>
+        <v>339.464</v>
       </c>
       <c r="J17" t="n">
-        <v>31107500000</v>
+        <v>31125600000</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1296,16 +1296,16 @@
         <v>44.7656</v>
       </c>
       <c r="F20" t="n">
-        <v>355.51</v>
+        <v>356.67</v>
       </c>
       <c r="G20" t="n">
-        <v>357.83</v>
+        <v>359.16</v>
       </c>
       <c r="H20" t="n">
-        <v>345.426</v>
+        <v>346.177</v>
       </c>
       <c r="I20" t="n">
-        <v>344.471</v>
+        <v>345.268</v>
       </c>
       <c r="J20" t="n">
         <v>11393400000</v>
@@ -1375,28 +1375,28 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>52.2164</v>
+        <v>52.2865</v>
       </c>
       <c r="D22" t="n">
         <v>20</v>
       </c>
       <c r="E22" t="n">
-        <v>42.6597</v>
+        <v>42.7438</v>
       </c>
       <c r="F22" t="n">
-        <v>354.4</v>
+        <v>364.1</v>
       </c>
       <c r="G22" t="n">
-        <v>356.26</v>
+        <v>371.4</v>
       </c>
       <c r="H22" t="n">
-        <v>351.288</v>
+        <v>333.773</v>
       </c>
       <c r="I22" t="n">
-        <v>351.445</v>
+        <v>333.229</v>
       </c>
       <c r="J22" t="n">
-        <v>108753000</v>
+        <v>53270600000</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1419,28 +1419,28 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>52.2411</v>
+        <v>52.7449</v>
       </c>
       <c r="D23" t="n">
-        <v>20.0531</v>
+        <v>20</v>
       </c>
       <c r="E23" t="n">
-        <v>42.8568</v>
+        <v>43.2939</v>
       </c>
       <c r="F23" t="n">
         <v>356.29</v>
       </c>
       <c r="G23" t="n">
-        <v>357.28</v>
+        <v>358.56</v>
       </c>
       <c r="H23" t="n">
         <v>346.162</v>
       </c>
       <c r="I23" t="n">
-        <v>345.295</v>
+        <v>345.32</v>
       </c>
       <c r="J23" t="n">
-        <v>7428300000</v>
+        <v>7450060000</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1472,16 +1472,16 @@
         <v>42.4896</v>
       </c>
       <c r="F24" t="n">
-        <v>354.08</v>
+        <v>356.41</v>
       </c>
       <c r="G24" t="n">
-        <v>355.79</v>
+        <v>358.51</v>
       </c>
       <c r="H24" t="n">
-        <v>351.286</v>
+        <v>352.135</v>
       </c>
       <c r="I24" t="n">
-        <v>351.432</v>
+        <v>352.392</v>
       </c>
       <c r="J24" t="n">
         <v>226227000</v>
@@ -1595,28 +1595,28 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>51.9886</v>
+        <v>51.3903</v>
       </c>
       <c r="D27" t="n">
         <v>20</v>
       </c>
       <c r="E27" t="n">
-        <v>42.3863</v>
+        <v>41.6684</v>
       </c>
       <c r="F27" t="n">
-        <v>355.16</v>
+        <v>358.28</v>
       </c>
       <c r="G27" t="n">
-        <v>357.29</v>
+        <v>362.28</v>
       </c>
       <c r="H27" t="n">
-        <v>332.4</v>
+        <v>334.226</v>
       </c>
       <c r="I27" t="n">
-        <v>331.573</v>
+        <v>333.295</v>
       </c>
       <c r="J27" t="n">
-        <v>59637200000</v>
+        <v>88812600000</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>

</xml_diff>